<commit_message>
Say 308, because that is what the server sends
Vercel answers permanent: true with a 308, not a 301. Google treats the
two the same, but the sheet goes to an SEO team who will check the code
against what it claims, so it should claim the right one.
</commit_message>
<xml_diff>
--- a/Portabox-SEO-Build-Sheet (updated).xlsx
+++ b/Portabox-SEO-Build-Sheet (updated).xlsx
@@ -7362,12 +7362,12 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t>DONE — merged into its region hub. The hub already covers this ground, so the old URL 301s to /self-storage/melbourne/ rather than running a second page against it.</t>
+          <t>DONE — merged into its region hub. The hub already covers this ground, so the old URL permanently redirects to /self-storage/melbourne/ rather than running a second page against it.</t>
         </is>
       </c>
     </row>
@@ -7410,12 +7410,12 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/melbourne/mornington/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Mornington, Melbourne, Victoria, 3931, Australia — 61 km by road from the Melbourne depot at Laverton North.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/melbourne/mornington/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Mornington, Melbourne, Victoria, 3931, Australia — 61 km by road from the Melbourne depot at Laverton North.</t>
         </is>
       </c>
     </row>
@@ -7458,12 +7458,12 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/sydney/penrith/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Penrith, Sydney, New South Wales, 2750, Australia — 25 km by road from the Sydney depot at Blacktown.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/sydney/penrith/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Penrith, Sydney, New South Wales, 2750, Australia — 25 km by road from the Sydney depot at Blacktown.</t>
         </is>
       </c>
     </row>
@@ -7506,12 +7506,12 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/gold-coast/burleigh/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Burleigh Heads, Gold Coast, Queensland, Australia — 56 km by road from the Brisbane depot at Gilberton.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/gold-coast/burleigh/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Burleigh Heads, Gold Coast, Queensland, Australia — 56 km by road from the Brisbane depot at Gilberton.</t>
         </is>
       </c>
     </row>
@@ -7554,12 +7554,12 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/melbourne/port-melbourne/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Port Melbourne, Melbourne, Victoria, 3207, Australia — 13 km by road from the Melbourne depot at Laverton North.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/melbourne/port-melbourne/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Port Melbourne, Melbourne, Victoria, 3207, Australia — 13 km by road from the Melbourne depot at Laverton North.</t>
         </is>
       </c>
     </row>
@@ -7650,12 +7650,12 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/melbourne/south-melbourne/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: South Melbourne, Melbourne, Victoria, 3205, Australia — 18 km by road from the Melbourne depot at Laverton North.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/melbourne/south-melbourne/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: South Melbourne, Melbourne, Victoria, 3205, Australia — 18 km by road from the Melbourne depot at Laverton North.</t>
         </is>
       </c>
     </row>
@@ -7698,12 +7698,12 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/melbourne/tullamarine/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Tullamarine, Melbourne, Victoria, 3043, Australia — 19 km by road from the Melbourne depot at Laverton North.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/melbourne/tullamarine/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Tullamarine, Melbourne, Victoria, 3043, Australia — 19 km by road from the Melbourne depot at Laverton North.</t>
         </is>
       </c>
     </row>
@@ -7746,12 +7746,12 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/melbourne/moorabbin/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Moorabbin, Melbourne, Victoria, 3189, Australia — 33 km by road from the Melbourne depot at Laverton North.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/melbourne/moorabbin/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Moorabbin, Melbourne, Victoria, 3189, Australia — 33 km by road from the Melbourne depot at Laverton North.</t>
         </is>
       </c>
     </row>
@@ -7794,12 +7794,12 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/brisbane/yatala/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Yatala, Logan City, Queensland, 4207, Australia — 8 km by road from the Brisbane depot at Gilberton.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/brisbane/yatala/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Yatala, Logan City, Queensland, 4207, Australia — 8 km by road from the Brisbane depot at Gilberton.</t>
         </is>
       </c>
     </row>
@@ -7842,12 +7842,12 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/brisbane/capalaba/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Capalaba, Logan City, Brisbane, Redland City, Queensland, Australia — 32 km by road from the Brisbane depot at Gilberton.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/brisbane/capalaba/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Capalaba, Logan City, Brisbane, Redland City, Queensland, Australia — 32 km by road from the Brisbane depot at Gilberton.</t>
         </is>
       </c>
     </row>
@@ -7890,12 +7890,12 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/sydney/north-sydney/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: North Sydney, New South Wales, 2060, Australia — 37 km by road from the Sydney depot at Blacktown.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/sydney/north-sydney/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: North Sydney, New South Wales, 2060, Australia — 37 km by road from the Sydney depot at Blacktown.</t>
         </is>
       </c>
     </row>
@@ -7938,12 +7938,12 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>DONE — dropped as a service page. Fremantle is in WA and the nearest depot is Adelaide, well past the 200 km standard-delivery range, so a page promising service there would not be true. The old URL 301s to /locations/regional-australia/, which is where a WA enquiry should land.</t>
+          <t>DONE — dropped as a service page. Fremantle is in WA and the nearest depot is Adelaide, well past the 200 km standard-delivery range, so a page promising service there would not be true. The old URL permanently redirects to /locations/regional-australia/, which is where a WA enquiry should land.</t>
         </is>
       </c>
     </row>
@@ -7986,12 +7986,12 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P113" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/sydney/brookvale/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Brookvale, Northern Beaches, Sydney, New South Wales, Australia — 43 km by road from the Sydney depot at Blacktown.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/sydney/brookvale/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Brookvale, Northern Beaches, Sydney, New South Wales, Australia — 43 km by road from the Sydney depot at Blacktown.</t>
         </is>
       </c>
     </row>
@@ -8034,12 +8034,12 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/sydney/marrickville/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Marrickville, Inner West, Sydney, New South Wales, 2204, Australia — 36 km by road from the Sydney depot at Blacktown.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/sydney/marrickville/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Marrickville, Inner West, Sydney, New South Wales, 2204, Australia — 36 km by road from the Sydney depot at Blacktown.</t>
         </is>
       </c>
     </row>
@@ -8082,12 +8082,12 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t>DONE — merged, not rebuilt. "Eastern Suburbs" is a region, not a suburb, so there is nothing to geocode and no single page it maps to. The old URL 301s to /self-storage/sydney/, which lists every Sydney suburb page beneath it, Bondi Junction among them.</t>
+          <t>DONE — merged, not rebuilt. "Eastern Suburbs" is a region, not a suburb, so there is nothing to geocode and no single page it maps to. The old URL permanently redirects to /self-storage/sydney/, which lists every Sydney suburb page beneath it, Bondi Junction among them.</t>
         </is>
       </c>
     </row>
@@ -8178,12 +8178,12 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/wollongong/unanderra/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Unanderra, Wollongong, New South Wales, Australia — 97 km by road from the Sydney depot at Blacktown.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/wollongong/unanderra/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Unanderra, Wollongong, New South Wales, Australia — 97 km by road from the Sydney depot at Blacktown.</t>
         </is>
       </c>
     </row>
@@ -8226,12 +8226,12 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/melbourne/north-melbourne/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: North Melbourne, Melbourne, Victoria, 3051, Australia — 16 km by road from the Melbourne depot at Laverton North.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/melbourne/north-melbourne/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: North Melbourne, Melbourne, Victoria, 3051, Australia — 16 km by road from the Melbourne depot at Laverton North.</t>
         </is>
       </c>
     </row>
@@ -8274,12 +8274,12 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/brisbane/chermside/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Chermside, Brisbane, Queensland, 4032, Australia — 58 km by road from the Brisbane depot at Gilberton.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/brisbane/chermside/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Chermside, Brisbane, Queensland, 4032, Australia — 58 km by road from the Brisbane depot at Gilberton.</t>
         </is>
       </c>
     </row>
@@ -8322,12 +8322,12 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/sydney/gladesville/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Gladesville, Sydney, New South Wales, 2111, Australia — 27 km by road from the Sydney depot at Blacktown.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/sydney/gladesville/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Gladesville, Sydney, New South Wales, 2111, Australia — 27 km by road from the Sydney depot at Blacktown.</t>
         </is>
       </c>
     </row>
@@ -8370,12 +8370,12 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/melbourne/altona/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Altona, Melbourne, Victoria, 3018, Australia — 5 km by road from the Melbourne depot at Laverton North.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/melbourne/altona/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Altona, Melbourne, Victoria, 3018, Australia — 5 km by road from the Melbourne depot at Laverton North.</t>
         </is>
       </c>
     </row>
@@ -8418,12 +8418,12 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P122" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/gold-coast/ormeau/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Ormeau, Queensland, Australia — 8 km by road from the Brisbane depot at Gilberton.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/gold-coast/ormeau/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Ormeau, Queensland, Australia — 8 km by road from the Brisbane depot at Gilberton.</t>
         </is>
       </c>
     </row>
@@ -8466,12 +8466,12 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P123" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/brisbane/aspley/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Aspley, Brisbane, Queensland, Australia — 62 km by road from the Brisbane depot at Gilberton.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/brisbane/aspley/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Aspley, Brisbane, Queensland, Australia — 62 km by road from the Brisbane depot at Gilberton.</t>
         </is>
       </c>
     </row>
@@ -8514,12 +8514,12 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P124" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/brisbane/brendale/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Brendale, Brisbane, Queensland, Australia — 70 km by road from the Brisbane depot at Gilberton.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/brisbane/brendale/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Brendale, Brisbane, Queensland, Australia — 70 km by road from the Brisbane depot at Gilberton.</t>
         </is>
       </c>
     </row>
@@ -8610,12 +8610,12 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/sydney/rozelle/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Rozelle, Inner West, Sydney, New South Wales, 2039, Australia — 34 km by road from the Sydney depot at Blacktown.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/sydney/rozelle/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Rozelle, Inner West, Sydney, New South Wales, 2039, Australia — 34 km by road from the Sydney depot at Blacktown.</t>
         </is>
       </c>
     </row>
@@ -8658,12 +8658,12 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>Live (301)</t>
+          <t>Live (308 redirect)</t>
         </is>
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>DONE — rebuilt, not migrated as-is. The old URL 301s to /self-storage/sydney/balmain/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Balmain, Inner West, Sydney, New South Wales, 2041, Australia — 34 km by road from the Sydney depot at Blacktown.</t>
+          <t>DONE — rebuilt, not migrated as-is. The old URL permanently redirects to /self-storage/sydney/balmain/, a suburb page written from scratch. Which hub it belongs under was settled by geocoding the name: Balmain, Inner West, Sydney, New South Wales, 2041, Australia — 34 km by road from the Sydney depot at Blacktown.</t>
         </is>
       </c>
     </row>

</xml_diff>